<commit_message>
Broaden job sources and redesign role discovery with company watchlists
</commit_message>
<xml_diff>
--- a/topics/job-search-agent/app/public/data/internships.xlsx
+++ b/topics/job-search-agent/app/public/data/internships.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internships" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company watchlist" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$W$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$Y$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$F$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Company watchlist'!$A$1:$M$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W14"/>
+  <dimension ref="A1:Y21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -471,6 +473,8 @@
     <col width="27" customWidth="1" min="21" max="21"/>
     <col width="27" customWidth="1" min="22" max="22"/>
     <col width="27" customWidth="1" min="23" max="23"/>
+    <col width="27" customWidth="1" min="24" max="24"/>
+    <col width="27" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
@@ -486,105 +490,115 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Role type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Work mode</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Minimum INR/month</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Maximum INR/month</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Pay confirmed in original</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Next action</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Interview time</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Applied date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Original source</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Application link</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Application email</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Application route</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Evidence / caveats</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Requirements</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Application instructions</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Posted</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>First discovered</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Last checked</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Personal notes</t>
         </is>
@@ -603,83 +617,93 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Remote, India</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>30000</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>30000</v>
       </c>
-      <c r="G2" s="2" t="b">
+      <c r="G2" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>discovered</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn job</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/jobs/view/ui-ux-design-intern-at-shramiksathi-4469701295</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>mailto:info@shramiksathi.com</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>info@shramiksathi.com</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Email application; draft can be prepared</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Employer-authored LinkedIn description explicitly states Remote (India) and ₹30,000/month. The job header says Bengaluru; the description confirms remote work. One opening listed.</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Figma, reusable components, design tokens, responsive and accessible interfaces, research and Hindi/English communication. Work includes worker-facing mobile flows and administrative dashboards. Internship: 3–6 months.</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Email a portfolio with 2–3 case studies and a response of up to 150 words: how should a worker confirm yesterday’s attendance on a small Android phone with an intermittent connection? No cover letter requested. Selection mentions a portfolio discussion, then a paid exercise.</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>3 weeks ago when checked</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="95" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -694,79 +718,89 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Ahmedabad, Gujarat</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>25000</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>30000</v>
       </c>
-      <c r="G3" s="2" t="b">
+      <c r="H3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>discovered</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>https://www.menstrupedia.com/careers/ux-intern</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>https://forms.gle/fWuuGCFJwACS7uVa9</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>Company application form</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>Company career page states internship, Ahmedabad office and ₹25,000–₹30,000/month. Meets the Gujarat minimum. Original posting date is not stated; confirm the opening is still available.</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Design web/mobile interfaces, test with users, collaborate with developers and measure outcomes. Visual design, typography, colour and English communication required. Past UX experience is desirable.</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>Use the company’s Apply link. The page also asks for a résumé and a paragraph explaining suitability, with subject Application for UX Design Intern.</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="V3" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr">
+      <c r="X3" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="95" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -781,75 +815,85 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>Bengaluru, Karnataka</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>35000</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>35000</v>
       </c>
-      <c r="G4" s="2" t="b">
+      <c r="G4" s="2" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>discovered</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn job</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/jobs/view/product-design-intern-at-more-retail-private-limited-4477072502</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/jobs/view/product-design-intern-at-more-retail-private-limited-4477072502</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>LinkedIn application</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>Employer-authored LinkedIn description states ₹35,000/month and Bengaluru. Remote work is not confirmed. Third-party ₹40,000 claims were not used.</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Portfolio showing design decisions and process, Figma, user research and design systems. Pursuing or recently completed a relevant design/HCI degree. Internship duration: 3–6 months.</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr">
         <is>
           <t>1 week ago when checked</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr">
+      <c r="X4" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="95" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -864,83 +908,93 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>Remote / hybrid, India</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Unconfirmed</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>20000</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>25000</v>
       </c>
-      <c r="G5" s="2" t="b">
+      <c r="H5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>discovered</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn job</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>https://in.linkedin.com/jobs/view/product-design-intern-at-bthree-design-agency-4473077505</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>mailto:contact@bthreedesigns.com</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>contact@bthreedesigns.com</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>Email application; draft can be prepared</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>Original listing gives ₹20,000–₹25,000/month and Remote / Hybrid. Conditional only if ₹25,000 is agreed and fully remote work is confirmed; the advertised minimum falls below your general threshold.</t>
-        </is>
-      </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Original listing gives ₹20,000–₹25,000/month and Remote / Hybrid. Conditional only if ₹25,000 is agreed and fully remote work is confirmed; the advertised minimum falls below your general threshold. An X mirror of the company post claims remote anywhere in India; original X access was blocked, so confirm with the employer.</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Strong Framer implementation, Figma auto-layout/components, design systems and motion tools such as Jitter or Lottie. Three-month internship, immediate start, eight hours/day.</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>Send portfolio/work samples, 2–3 lines on work you enjoy and 2–3 lines on what you want to learn. Framer/motion examples are useful.</t>
         </is>
       </c>
-      <c r="T5" s="2" t="inlineStr">
+      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>3 weeks ago when checked</t>
         </is>
       </c>
-      <c r="U5" s="2" t="inlineStr">
+      <c r="W5" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V5" s="2" t="inlineStr">
+      <c r="X5" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="95" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -955,71 +1009,81 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>Bengaluru, Karnataka</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="b">
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn post</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/posts/sruthisivakumar_product-design-intern-wint-wealth-activity-7515659430051426304-tqUQ</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>https://binary.so/P01RayN</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>Recruiter-linked application form</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>A current post by the company’s co-founder/design leader confirms the internship and Bangalore office attendance. ₹30k–₹35k appears only in third-party listings; employer pay is unconfirmed.</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>Figma, product thinking, collaboration with product and engineering. Portfolio work on design systems is specifically encouraged.</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr">
         <is>
           <t>1 week ago when checked</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr">
+      <c r="W6" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr">
+      <c r="X6" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="95" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1034,71 +1098,81 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>Bengaluru, Karnataka</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="b">
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/hevodata/433ffdef-3125-48ed-a131-52c697c321ee</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/hevodata/433ffdef-3125-48ed-a131-52c697c321ee/apply</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>Lever application form</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>Official employer Lever role and application page are accessible. On-site Bangalore; stipend and original publication date are not disclosed.</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>Figma components and tokens, SaaS/dashboard interfaces, prototyping and developer handoff. AI-assisted design workflows are relevant.</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr">
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="X7" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="95" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1113,71 +1187,81 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>Bengaluru, Karnataka</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>On-site</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="b">
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>https://www.revrag.ai/careers/product-design-intern</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>https://www.revrag.ai/careers/product-design-intern</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>Employer-linked Google Form</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>Original company role is accessible and lists Bengaluru on-site. Third-party ₹40k claims are not confirmed by this page.</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>Strong portfolio, Figma variables/components, AI prototyping, interaction states and fintech workflows. Six-month internship.</t>
         </is>
       </c>
-      <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr">
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="U8" s="2" t="inlineStr">
+      <c r="W8" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr">
+      <c r="X8" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="95" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1192,79 +1276,89 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>Remote, India; Bengaluru preferred</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="b">
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>https://chiblu.com/careers/product-design-intern-ux-ui</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>mailto:apply@chiblu.com</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>apply@chiblu.com</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>Email or Wellfound</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="inlineStr">
+      <c r="S9" s="2" t="inlineStr">
         <is>
           <t>Company still exposes the role page and links it from careers. It is an older May posting; current hiring and stipend require confirmation.</t>
         </is>
       </c>
-      <c r="R9" s="2" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>At least three portfolio projects, including end-to-end thinking and a mobile flow; Figma, visual craft, research and communication. Two months with possible extension.</t>
         </is>
       </c>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t>Share portfolio, a short reason for your interest, one project you would discuss and earliest start date.</t>
         </is>
       </c>
-      <c r="T9" s="2" t="inlineStr">
+      <c r="V9" s="2" t="inlineStr">
         <is>
           <t>5 May 2026 · older posting</t>
         </is>
       </c>
-      <c r="U9" s="2" t="inlineStr">
+      <c r="W9" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr">
+      <c r="X9" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W9" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="95" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1279,71 +1373,81 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>Remote, India</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="b">
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>https://www.neuralpath.app/careers/</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>https://www.neuralpath.app/careers/</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>Email application via company page</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="inlineStr">
+      <c r="S10" s="2" t="inlineStr">
         <is>
           <t>Company careers page explicitly lists a remote Product Design Intern opportunity and year-round applications. Duration and stipend are discussed individually.</t>
         </is>
       </c>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>Figma, UI, prototypes and a portfolio. Students/recent graduates welcome; internships can fit around classes.</t>
         </is>
       </c>
-      <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr">
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="U10" s="2" t="inlineStr">
+      <c r="W10" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr">
+      <c r="X10" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W10" s="2" t="inlineStr"/>
+      <c r="Y10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="95" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1358,71 +1462,81 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>Remote, India</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="b">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>https://krmrsolutions.com/careers/design-intern</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>https://krmrsolutions.com/careers/design-intern</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr">
         <is>
           <t>LinkedIn link from employer page</t>
         </is>
       </c>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="S11" s="2" t="inlineStr">
         <is>
           <t>Original company career page confirms Remote (India) and internship. No stipend or publication date stated.</t>
         </is>
       </c>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t>Portfolio showing layout, typography and colour; Figma auto-layout and prototypes; component documentation and development handoff.</t>
         </is>
       </c>
-      <c r="S11" s="2" t="inlineStr"/>
-      <c r="T11" s="2" t="inlineStr">
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="U11" s="2" t="inlineStr">
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr">
+      <c r="X11" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W11" s="2" t="inlineStr"/>
+      <c r="Y11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="95" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1437,71 +1551,81 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>Remote, India</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="b">
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>https://www.gozavio.com/careers</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>https://www.gozavio.com/careers</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t>Company application link</t>
         </is>
       </c>
-      <c r="Q12" s="2" t="inlineStr">
+      <c r="S12" s="2" t="inlineStr">
         <is>
           <t>Company careers page lists this as an open internship, remote anywhere in India. Stipend and posting date are not stated.</t>
         </is>
       </c>
-      <c r="R12" s="2" t="inlineStr">
+      <c r="T12" s="2" t="inlineStr">
         <is>
           <t>Research, wireframes, user flows and high-fidelity interfaces for financial education products.</t>
         </is>
       </c>
-      <c r="S12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="inlineStr">
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="U12" s="2" t="inlineStr">
+      <c r="W12" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr">
+      <c r="X12" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W12" s="2" t="inlineStr"/>
+      <c r="Y12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1516,71 +1640,81 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>Remote, India (reported)</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="b">
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Job board</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>https://www.jobleads.com/in/job/product-design-intern--india--e24abd61a6654a91f9a3af3bab3db8da5</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="P13" s="3" t="inlineStr">
         <is>
           <t>https://www.gnixar.in/careers</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>Confirm on employer careers first</t>
         </is>
       </c>
-      <c r="Q13" s="2" t="inlineStr">
+      <c r="S13" s="2" t="inlineStr">
         <is>
           <t>Job-board description reports remote India and ₹25k–₹40k/month, but its header conflicts on location and compensation. The company careers page dynamically loads roles; this role/pay remains unverified.</t>
         </is>
       </c>
-      <c r="R13" s="2" t="inlineStr">
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>Visual and interaction design portfolio, Figma, prototyping and design-system contributions.</t>
         </is>
       </c>
-      <c r="S13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="inlineStr">
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr">
         <is>
           <t>13 days ago on job board when checked</t>
         </is>
       </c>
-      <c r="U13" s="2" t="inlineStr">
+      <c r="W13" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V13" s="2" t="inlineStr">
+      <c r="X13" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W13" s="2" t="inlineStr"/>
+      <c r="Y13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="95" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1595,106 +1729,781 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>Bengaluru, Karnataka</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Unconfirmed</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="b">
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>discovered</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Job board</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>https://www.studentsmart.co.in/student/internships/glance-ux-design-intern</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>https://www.studentsmart.co.in/student/internships/glance-ux-design-intern</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr">
         <is>
           <t>Job-board sign-in; find original employer listing</t>
         </is>
       </c>
-      <c r="Q14" s="2" t="inlineStr">
+      <c r="S14" s="2" t="inlineStr">
         <is>
           <t>StudentSmart reports ₹30k–₹40k/month and Bengaluru; original employer confirmation and work arrangement are still needed.</t>
         </is>
       </c>
-      <c r="R14" s="2" t="inlineStr">
+      <c r="T14" s="2" t="inlineStr">
         <is>
           <t>UX/visual design for TV shopping interfaces, design systems, interaction states, engineering handoff and interest in AI/ambient computing.</t>
         </is>
       </c>
-      <c r="S14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="inlineStr">
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="inlineStr">
         <is>
           <t>15 October 2026 on job board</t>
         </is>
       </c>
-      <c r="U14" s="2" t="inlineStr">
+      <c r="W14" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="V14" s="2" t="inlineStr">
+      <c r="X14" s="2" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="W14" s="2" t="inlineStr"/>
+      <c r="Y14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="95" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Techolution</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad / remote claim requires confirmation</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Confirm current vacancy, India remote eligibility and at least ₹25–30k/month before submitting.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=e1a25a765d7c4fd7</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>https://hire.techolution.com/careers</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Indeed application or locate UX Designer–Intern on employer careers portal; form and account requirements untested</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>Indeed detail accessible; official careers index also lists UX Designer–Intern in Hyderabad. Remote statement in Indeed conflicts with Hyderabad in current company index. Official careers site is dynamic; indexed role corroboration is stronger than its text-only rendering.</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio and Figma; Interaction/UX/graphic design or related degree; Research, wireframes, prototypes and developer specifications.</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>No reliable original posting date displayed</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>F1studioz</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Ask stipend, Bengaluru attendance requirements and six-month availability before applying.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=fef929ca634359c7</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=fef929ca634359c7</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Indeed; official careers page provides careers@f1studioz.com as company hiring channel.</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>Original Indeed detail accessible without an expiry banner; official careers page corroborates employer and application channel, not a unique role detail. Actual application submission flow not tested. General company hybrid policy does not establish this role's work mode.</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>Practice projects accepted in portfolio; Final-semester B.Des/M.Des or engineering student/graduate with UX skills; AI tools and enterprise UX interest; possible full-time availability.</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="95" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Green Ping Solutions</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Confirm stipend of at least ₹20k/month and internship duration.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=157d2635900933e2</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=157d2635900933e2</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Indeed SmartApply</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>Original Indeed detail accessible without an expiry banner. Login and application fields not inspected through submission.</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>Web and mobile UI; User research, flows and prototypes; Components/design systems and developer collaboration.</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="95" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Moon Technolabs</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Trainee UI/UX Designer</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Confirm starting monthly salary ≥₹20k and graduate eligibility.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=45ad3491be217187</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moontechnolabs.com/career-with-us/</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Official careers Apply Now / career@moontechnolabs.com, or Indeed</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>Indeed detail accessible; official careers page lists Trainee UI/UX Designer with experience Fresher. Submission not tested; this is a junior job alternative, not an internship.</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Figma or Adobe XD; Wireframes, prototypes, research and design systems; Bachelor's graduate and developer handoff skills.</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Keyideas Infotech</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Remote India (confirm eligibility)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Verify active Naukri route and paid stipend ≥₹25–30k before investing in application.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Naukri</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-ui-ux-internship-figma-graphics-research-keyideas-infotech-gurgaon-gurugram-0-to-1-years-181120004352</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-ui-ux-internship-figma-graphics-research-keyideas-infotech-gurgaon-gurugram-0-to-1-years-181120004352</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Employer page directs applicants to Naukri; no WhatsApp applications.</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Current accessible employer role page explicitly links this Naukri application. Original Naukri page is robots-blocked, so activity of that particular Naukri listing is unverified. Employer says remote; Naukri slug says Gurgaon. Confirm remote India eligibility and current application link.</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>B.Des/M.Des or relevant design qualification; Figma and Illustrator; Research/usability, web/mobile design, components and brand styles.</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr"/>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>No reliable posting date. Naukri identifier appears historical; do not infer freshness.</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="95" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Zunderdog</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Pune; remote for now</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Remote for now</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Confirm paid stipend and whether eventual Pune attendance is required.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers/ui-ux-design-intern-pune</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers/ui-ux-design-intern-pune</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Employer form with resume, education, experience, notice period, location, expected salary and privacy consent.</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>Official role and application form accessible. Employer prefers candidates in or near Pune. Remote arrangement is temporary; no promise of permanent remote. Application form not submitted.</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>Figma basics; Few college, personal or professional design projects; Layout, wireframes, simple prototypes and checking developed screens.</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr"/>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>Careers index shows a relative age of 2 days; original absolute publication date not independently available.</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Zunderdog</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Designer (Fresher)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Pune; remote for now</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Remote for now</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Confirm salary ≥₹25–30k/month and future office expectations.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers/ui-ux-designer-fresher-pune</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers/ui-ux-designer-fresher-pune</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>Employer application form; resume, location, expected annual salary and privacy consent required.</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>Official role and application form accessible; Indeed discovery was a search result, not a uniquely verified job-detail URL. Employer prefers Pune or nearby candidates; current remote arrangement may change.</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Figma and portfolio; personal/college/freelance work accepted; Flows, prototypes, accessible UI and design systems; Developer collaboration and usability reviews.</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr"/>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>Careers index shows a relative age of 2 days; original absolute publication date not independently available.</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="Y21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W14"/>
+  <autoFilter ref="A1:Y21"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"discovered,shortlisted,applied,assessment,interview,offer,closed"</formula1>
+    <dataValidation sqref="I2:I10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"discovered,shortlisted,on_hold,applied,assessment,interview,offer,closed"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1706,7 +2515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2229,8 +3038,600 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Techolution</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=e1a25a765d7c4fd7</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>F1studioz</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=fef929ca634359c7</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Green Ping Solutions</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=157d2635900933e2</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Moon Technolabs</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>https://in.indeed.com/viewjob?jk=45ad3491be217187</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Keyideas Infotech</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-ui-ux-internship-figma-graphics-research-keyideas-infotech-gurgaon-gurugram-0-to-1-years-181120004352</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Zunderdog</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers/ui-ux-design-intern-pune</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Zunderdog</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers/ui-ux-designer-fresher-pune</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.microsoft.com/v2/global/en/students</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.adobe.com/us/en/university</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Atlassian</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.atlassian.com/company/careers/earlycareers</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Tekion</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>https://tekion.com/careers</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Scaler Academy</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/careers/</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Lenskart</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.lenskart.com/</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>ShramikSathi</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>https://shramiksathi.com/</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Rapido</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rapido.bike/Careers</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>SatSure</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.satsure.co/careers/</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>BThree Design Agency</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bthreedesigns.com/</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Parallel</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.parallelhq.com/careers</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>F1studioz</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>https://f1studioz.com/careers</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Moon Technolabs</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.moontechnolabs.com/career-with-us/</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Zunderdog</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Keyideas Infotech</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.keyideasinfotech.com/careers/ui-ux-design-internship/</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>careers</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Wint Wealth</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/beatsbyshaz/status/2112981756571983955</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>social</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Original X URL returned 403; content checked through third-party mirror. Evidence: https://workingww.twstalker.com/beatsbyshaz/status/2112981756571983955</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>BThree Designs</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/BThreeAgency/status/2108934891069161479</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>social</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Original X URL returned 403; content checked through third-party mirror. Evidence: https://workingww.twstalker.com/BThreeAgency/status/2108934891069161479</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2241,7 +3642,1170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="75" customWidth="1" min="4" max="4"/>
+    <col width="75" customWidth="1" min="5" max="5"/>
+    <col width="75" customWidth="1" min="6" max="6"/>
+    <col width="75" customWidth="1" min="7" max="7"/>
+    <col width="75" customWidth="1" min="8" max="8"/>
+    <col width="75" customWidth="1" min="9" max="9"/>
+    <col width="75" customWidth="1" min="10" max="10"/>
+    <col width="75" customWidth="1" min="11" max="11"/>
+    <col width="75" customWidth="1" min="12" max="12"/>
+    <col width="75" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="29" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Suggested category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Why this target</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pay evidence type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reported role</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Range minimum</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Range maximum</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Original period</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Limitations</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Careers URL</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Pay source</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Observed date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Dream</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Product-design teams across enterprise and consumer software. Keep India student and early-career openings on your radar.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Older, low-confidence UX intern reports with inconsistent geography. Current India stipend and eligibility need confirmation.</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.microsoft.com/v2/global/en/students</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Salary/Microsoft-UX-Design-intern-Bangalore-EJI_IE1651.0%2C9_KO10%2C26_IL.27%2C36_IM1091.htm?filter.payPeriod=MONTHLY</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Dream</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Creative tools and digital experience products. Watch India university and early-career design roles.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Modeled salary estimate</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>UI UX Design Intern</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>A related-designation salary model gives an annual intern estimate; exact India internship pay is not established. No monthly stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.adobe.com/us/en/university</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ambitionbox.com/salaries/adobe-salaries/ui-ux-architect</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Atlassian</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Dream</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Collaboration products and design systems. Watch for India-eligible early-career opportunities.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Only two annualized intern reports, with unclear geography. The current US internship found in research is not an India opportunity.</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.atlassian.com/company/careers/earlycareers</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>https://static.glassdoor.co.in/Salary/Atlassian-Salaries-E115699_P10.htm</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Tekion</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Suggested practical product-company target with direct design-intern salary history, not a hiring probability.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>46000</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>72000</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Historical small sample; source labels low confidence. Current stipend, role availability and remote eligibility need employer confirmation.</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>https://tekion.com/careers</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Salary/Tekion-Product-Design-Intern-Bangalore-Salaries-EJI_IE1501014.0%2C6_KO7%2C28_IL.29%2C38_IM1091.htm?payPeriod=MONTHLY</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Scaler Academy</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Suggested product-design target with reported internship compensation near the requested ballpark.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>28000</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Old employee reports, not a current offer. Careers page currently exposes other roles; no matching internship confirmed.</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.scaler.com/careers/</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Salary/Scaler-Academy-Product-Design-Intern-Bengaluru-Salaries-EJI_IE3340290.0%2C14_KO15%2C36_IL.37%2C46_IC2940587.htm?payPeriod=MONTHLY</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Lenskart</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Suggested consumer-product employer with a design-intern salary signal.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>39000</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>42000</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>One report, location/date of report not shown. Official careers redirects to a company job board displaying0 jobs on24 Oct2026; watchlist only.</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.lenskart.com/</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>https://static.glassdoor.co.in/Salary/Lenskart-Solutions-Salaries-E742328_P56.htm</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Menstrupedia</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Suggested practical target because its employer-stated internship range meets the Gujarat minimum.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Employer-listed stipend</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Employer-listed</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Listing publication date absent; an accessible page does not guarantee recruitment is still open.</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.menstrupedia.com/careers/ux-intern</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.menstrupedia.com/careers/ux-intern</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ShramikSathi</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Suggested practical target with explicit remote internship pay and concrete product-design responsibilities.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Employer-listed stipend</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Employer-listed snapshot</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Employer website is verified, but no separate careers page was located. Listing freshness should be reconfirmed; source is an employer-authored LinkedIn job, not a current employee pay report.</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>https://shramiksathi.com/</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/ui-ux-design-intern-at-shramiksathi-4469701295</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Rapido</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Suggested exploratory product-design target; reported pay spans below and above the requested minimum.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>38000</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Small sample with substantial variation; not enough to assume all internships meet INR30k. Source labels low confidence.</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rapido.bike/Careers</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Salary/Rapido-Product-Design-Intern-Bangalore-Salaries-EJI_IE1150759.0%2C6_KO7%2C28_IL.29%2C38_IM1091.htm?payPeriod=MONTHLY</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SatSure</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Suggested exploratory B2B/geospatial-product target with design-intern salary history near the conditional band.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Annualized salary display is not a confirmed internship-term payment. INR25k/month is only arithmetic annual/12 equivalence; current amount and duration must be checked.</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.satsure.co/careers/</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.glassdoor.co.in/Salary/SatSure-Salaries-E4629454_P2.htm</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>BThree Design Agency</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Suggested exploratory studio target; advertised maximum reaches the user’s conditional INR25k band.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Employer-listed stipend</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Employer-listed snapshot</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Below general minimum unless INR25k is agreed. Verify work mode and whether the role remains open. Company website verified; separate careers page not found.</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bthreedesigns.com/</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/product-design-intern-at-bthree-design-agency-4473077505</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Parallel</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Suggested exploratory specialist-studio target with remote design work; pay range overlaps the conditional band.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Third-party listing</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Treat as historical/unverified rather than a live job. Official careers page is accessible but did not independently confirm this internship or stipend.</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.parallelhq.com/careers</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>https://jobgether.com/offer/6a88dfb41de6f4542a4decc5-product-design-intern</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>F1studioz</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise UX studio with a current intern listing, but historical internship pay is below your target. Confirm the current budget before applying.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Low-confidence page displays about ₹10k/month and5 submissions, updated4 June2025. Historical report is below your target; verify whether this current role has a different budget.</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>https://f1studioz.com/careers</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Monthly-Pay/f1Studioz-UX-Intern-Remote-India-Monthly-Pay-EJI_IE1588351.0%2C9_KO10%2C19_IL.20%2C32_IS12563.htm</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Moon Technolabs</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Employer careers lists a fresher UI/UX trainee role in Gujarat. Confirm starting pay and graduate requirements.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Current posting does not disclose pay. No reliable role-specific salary estimate was established in this research pass.</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moontechnolabs.com/career-with-us/</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Zunderdog</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Official intern and fresher roles accept personal or college projects. Confirm stipend and eventual Pune attendance.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Current posting does not disclose pay. No reliable role-specific salary estimate was established in this research pass.</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zunderdog.com/careers</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Keyideas Infotech</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Employer page lists a remote UI/UX internship and links to Naukri. Check whether the historical application route is still active.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>UI UX Design Intern</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>19000</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Cross-company salary page reports ₹19k–₹21k/month for Keyideas in New Delhi. Sample/date unavailable and location differs from the remote posting. This is below the general target and does not establish current pay.</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.keyideasinfotech.com/careers/ui-ux-design-internship/</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.com/Salaries/ui-ux-design-intern-salary-SRCH_IM1083_KO0%2C19_P4.htm</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Techolution</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>UX internship listings and historical pay near the conditional range. Confirm remote eligibility and the current stipend first.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Reported salary</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>29000</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Historical reports</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Visible reports range from ₹15k in May2024 to ₹25k–₹29k in2025. The page also models ₹18k–₹30k/month across10 submissions. Reports are not the current role’s offer; confirm ₹25k–₹30k and remote terms.</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>https://hire.techolution.com/careers</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/Salary/Techolution-UX-Design-intern-India-Salaries-EJI_IE1397522.0%2C11_KO12%2C28_IL.29%2C34_IN115.htm?payPeriod=MONTHLY</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M18"/>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Dream,Workable,Possible"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId32"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2256,7 +4820,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Research snapshot: 2026-10-23</t>
+          <t>Research snapshot: 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -2292,151 +4856,247 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Only employer-stated minimums count as confirmed. Undisclosed and third-party pay must be checked.</t>
+          <t>Only employer-stated minimums count as confirmed. Undisclosed-pay roles stay on hold. Glassdoor and other company reports are historical context, never a current offer. Annual figures stay annual.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Freshness</t>
+          <t>Company groups</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Discovery date is not posting date. An accessible listing does not guarantee current hiring.</t>
+          <t>Dream / Workable / Possible are editable suggestions, not hiring probabilities. The company watchlist does not assert current vacancies or offers.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Applications</t>
+          <t>Freshness</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>No applications have been submitted. Status and application fields are for you to update.</t>
+          <t>Discovery date is not posting date. An accessible listing does not guarantee current hiring.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Board vs Excel</t>
+          <t>Applications</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>This workbook contains the research snapshot. Browser board changes are exported separately using CSV or JSON backup.</t>
+          <t>No applications have been submitted. Status and application fields are for you to update.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Privacy</t>
+          <t>Board vs Excel</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Initial workbook contains no résumé or personal contact data. Employer application contacts are public listing details.</t>
+          <t>This workbook contains the research snapshot. Browser board changes are exported separately using CSV or JSON backup.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Excluded roles</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>See the exclusion list below.</t>
+          <t>Initial workbook contains no résumé or personal contact data. Employer application contacts are public listing details.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Appbrew</t>
+          <t>Excluded roles</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Previously indexed Wellfound role returned HTTP 410 Gone; excluded as an active opening.</t>
+          <t>See the exclusion list below.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Parallel</t>
+          <t>Appbrew</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Third-party role returned HTTP 410 Gone. General careers page alone does not confirm an internship or stipend.</t>
+          <t>Previously indexed Wellfound role returned HTTP 410 Gone; excluded as an active opening.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CrossBo</t>
+          <t>Parallel</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Remote recruiter post is approximately seven months old; stipend and current hiring not confirmed.</t>
+          <t>Third-party role returned HTTP 410 Gone. General careers page alone does not confirm an internship or stipend.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Ourora</t>
+          <t>CrossBo</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Remote internship is explicitly unpaid and falls below your stipend requirements.</t>
+          <t>Remote recruiter post is approximately seven months old; stipend and current hiring not confirmed.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Trinance</t>
+          <t>Ourora</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad on-site internship lists ₹20,000/month, below your non-Gujarat minimum.</t>
+          <t>Remote internship is explicitly unpaid and falls below your stipend requirements.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>hussh Pune</t>
+          <t>Trinance</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Stale snippet advertises ₹40k, but the current page gives no stipend and describes a campus challenge/probation process; keep outside confirmed matches.</t>
+          <t>Hyderabad on-site internship lists ₹20,000/month, below your non-Gujarat minimum.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>hussh Pune</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Searched public indexed hiring posts; no independently verified qualifying original post found in this pass.</t>
+          <t>Stale snippet advertises ₹40k, but the current page gives no stipend and describes a campus challenge/probation process; keep outside confirmed matches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>DronaHQ</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Original Indeed detail explicitly says expired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>iVoyant</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Original Indeed result explicitly says expired; another listing 0d6b9d4b3f8986b1 also expired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Zuntra Digital</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Official employer description explicitly says unpaid 3-month internship; old Naukri-associated salary snippets must not override this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>SurveySparrow</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Indeed lists ₹10,000–20,000 a year, not a month. Below threshold as written; do not silently change unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>FX31Labs</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Naukri-associated identifier appears old; aggregator result is unrelated head role with another-card snippet. Official career page did not verify active internship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Kevit.io</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Indexed Naukri-associated lead is historical and current original Naukri/employer vacancy could not be established. Avoid presenting as newly active Naukri role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TensorGo</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Indeed detail remains accessible, but original company role returns HTTP 410 Gone. Company-side deletion conflicts with accessible Indeed listing; do not label verified active.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>CartGeek</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Indeed and employer page accessible. Another employer posting on LinkedIn categorizes the same title as Volunteer; paid status is not established. Possible volunteer/unpaid classification; do not recommend as a qualifying paid role until clarified.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh design job research for 25 October and archive removed listing
</commit_message>
<xml_diff>
--- a/topics/job-search-agent/app/public/data/internships.xlsx
+++ b/topics/job-search-agent/app/public/data/internships.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$Z$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$F$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$Z$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$F$256</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source coverage'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Company watchlist'!$A$1:$M$116</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Company directory'!$A$1:$M$116</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Role requirements'!$A$1:$I$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Company watchlist'!$A$1:$M$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Company directory'!$A$1:$M$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Role requirements'!$A$1:$I$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -811,7 +811,7 @@
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr"/>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z7" s="2" t="inlineStr"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
-          <t>Company still exposes the role page and links it from careers. It is an older May posting; current hiring and stipend require confirmation.</t>
+          <t>Company still exposes the role page and links it from careers. It is an older May posting; current hiring and stipend require confirmation. Recheck25 October: employer page remains accessible; linked Wellfound4209561 now returns410 Gone. The employer page alone does not establish a renewed intake.</t>
         </is>
       </c>
       <c r="U9" s="2" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr"/>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z10" s="2" t="inlineStr"/>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr"/>
@@ -1777,34 +1777,38 @@
           <t>on_hold</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Confirm stipend, office arrangement, duration and start window via the official role.</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Job board</t>
+          <t>Company careers</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>https://www.studentsmart.co.in/student/internships/glance-ux-design-intern</t>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>https://www.studentsmart.co.in/student/internships/glance-ux-design-intern</t>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Job-board sign-in; find original employer listing</t>
+          <t>Official Greenhouse application</t>
         </is>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>StudentSmart reports ₹30k–₹40k/month and Bengaluru; original employer confirmation and work arrangement are still needed.</t>
+          <t>Original Glance Greenhouse role and application are available. Stipend is not stated; the prior StudentSmart INR30–40k/month claim remains unverified. Confirm work arrangement and start date.</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -1815,7 +1819,7 @@
       <c r="V14" s="2" t="inlineStr"/>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>15 October 2026 on job board</t>
+          <t>Employer date unstated; 15 October was the aggregator date</t>
         </is>
       </c>
       <c r="X14" s="2" t="inlineStr">
@@ -1825,7 +1829,7 @@
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z14" s="2" t="inlineStr"/>
@@ -1919,7 +1923,7 @@
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr"/>
@@ -2013,7 +2017,7 @@
       </c>
       <c r="Y16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z16" s="2" t="inlineStr"/>
@@ -2107,7 +2111,7 @@
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z17" s="2" t="inlineStr"/>
@@ -2201,7 +2205,7 @@
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z18" s="2" t="inlineStr"/>
@@ -2577,7 +2581,7 @@
       </c>
       <c r="Y22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z22" s="2" t="inlineStr"/>
@@ -2765,7 +2769,7 @@
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z24" s="2" t="inlineStr"/>
@@ -2859,7 +2863,7 @@
       </c>
       <c r="Y25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z25" s="2" t="inlineStr"/>
@@ -3448,7 +3452,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Intern - UI/UX / Web Designer</t>
+          <t>Intern-UI/UX</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3512,7 +3516,7 @@
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>Indeed detail publicly opened. Three-month UI/UX and web/landing-page internship, in person in Mumbai. Employer careers page confirms company and publishes general HR contact, but this internship was not visible in extracted official openings. Pay/current intake unconfirmed.</t>
+          <t>Indeed detail publicly opened. Three-month UI/UX and web/landing-page internship, in person in Mumbai. Employer careers page confirms company and publishes general HR contact, but this internship was not visible in extracted official openings. Pay/current intake unconfirmed. Original detail now uses Intern-UI/UX; stable record ID preserved.</t>
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr">
@@ -3533,7 +3537,7 @@
       </c>
       <c r="Y32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z32" s="2" t="inlineStr"/>
@@ -3994,7 +3998,7 @@
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t>Himalayas detail and documented public API both accessible; API per-job check returned200. Detail explicitly permits all countries and API has no country restrictions plus UTC+05:30. Original company site was opened but only ASO/User Acquisition roles were visible, so the UX vacancy is not corroborated on its site. Pay undisclosed. Board labels entry-level while body requires1–2 commercial years.</t>
+          <t>Himalayas detail and documented public API both accessible; API per-job check returned200. Detail explicitly permits all countries and API has no country restrictions plus UTC+05:30. Original company site was opened but only ASO/User Acquisition roles were visible, so the UX vacancy is not corroborated on its site. Pay undisclosed. Board labels entry-level while body requires1–2 commercial years. Recheck25 October: board detail still gives5 November deadline. Job expired? is a reporting control, not a closure notice.</t>
         </is>
       </c>
       <c r="U37" s="2" t="inlineStr">
@@ -4015,7 +4019,7 @@
       </c>
       <c r="Y37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z37" s="2" t="inlineStr"/>
@@ -4148,12 +4152,12 @@
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>on_hold</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Confirm current paid employment intake, no applicant fees, India eligibility, duration/start window and remote stipend around INR30,000/month; INR25,000 only considered individually.</t>
+          <t>Archived: original role removed. Reopen only when a current employer vacancy is evidenced.</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -4182,7 +4186,7 @@
       </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation.</t>
+          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation. Recheck25 October: original role returned404 in direct check and410 Gone through web research. Archived as a removed listing; no claim that all company hiring ended.</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
@@ -4203,7 +4207,7 @@
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Z39" s="2" t="inlineStr"/>
@@ -4302,8 +4306,392 @@
       </c>
       <c r="Z40" s="2" t="inlineStr"/>
     </row>
+    <row r="41" ht="95" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Remote within India; Gurugram office optional/preferred</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Confirm monthly stipend, internship duration and start window; review the portfolio request.</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern/apply</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr"/>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS/form; manual review and submission</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>Employer detail and application page are available; the form explicitly permits work from home within India. Duration, stipend amount and cohort/start dates are unstated. General employee perks are not confirmed intern benefits.</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>Figma proficiency and a portfolio showing design reasoning; Interface fundamentals, interaction flows and usability; Independent ownership and collaboration with engineering; Interest in AI creative tools; prior product work is optional</t>
+        </is>
+      </c>
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr">
+        <is>
+          <t>12 October 2026 in employer JobPosting metadata</t>
+        </is>
+      </c>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="95" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Thane / Mumbai, Maharashtra; employer pages use both locations</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Confirm stipend, duration, office location and start date with the official listing; complete both required steps only after review.</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>https://revvity.wd103.myworkdayjobs.com/External/job/Mumbai/UX-Intern_JR-045767/apply</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr"/>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS/form; manual review and submission</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Official careers detail lists JR-045767 and links the Workday application plus a mandatory Microsoft questionnaire. Both steps are required. Workday was not accessible through the research tool; no submission flow tested. Unstop lists 5 November while another mirror gives 7 December; neither is an employer-confirmed deadline.</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>Awareness of UX design and research methods; Clear English communication and presenting design decisions; Curiosity, feedback and collaboration; Work includes prototyping and research sessions</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="inlineStr">
+        <is>
+          <t>The employer requires its questionnaire https://forms.cloud.microsoft/r/agdKBU4dTM and submission to Workday for JR-045767. Review both before sending anything.</t>
+        </is>
+      </c>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t>8 October 2026 in official careers structured data; mirror dates differ</t>
+        </is>
+      </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="95" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>UI / UX Design Trainee (Fresher)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>INR 250000–400000/year</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Confirm full-time eligibility, joining window and annual package; use the paid-job ATS route, not training programs.</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/apply.php?job_id=50</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr"/>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS/form; manual review and submission</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS and corporate careers page corroborate this paid job. Unpaid training programs are separate and excluded. Apply through ATS only; the support address is technical support, not a recruitment inbox. Start timing and employment terms need confirmation.</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>Design, HCI, fine-arts or related qualification; Working Figma knowledge and a portfolio; coursework is accepted; Wireframes, design-system components and research support; Openness to critique</t>
+        </is>
+      </c>
+      <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="inlineStr">
+        <is>
+          <t>19 September 2026 on original employer detail</t>
+        </is>
+      </c>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y43" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="95" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>UI Designer – 0–1 Years Experience</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Confirm salary, student/graduate eligibility, later joining and actual office schedule before applying.</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="R44" s="2" t="inlineStr"/>
+      <c r="S44" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS/form; manual review and submission</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>0–1 years; graduates with a portfolio are welcome; Figma and strong typography, spacing, grids and interface hierarchy; Basic UX knowledge and responsive SaaS interfaces; Collaboration, iteration and curiosity about AI tools; Bonus: design systems, HTML/CSS and prior design internship</t>
+        </is>
+      </c>
+      <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="inlineStr">
+        <is>
+          <t>Original posting date unstated; update age is not a publication date</t>
+        </is>
+      </c>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y44" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z44" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z40"/>
+  <autoFilter ref="A1:Z44"/>
   <dataValidations count="1">
     <dataValidation sqref="J2:J10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"discovered,shortlisted,on_hold,applied,assessment,interview,offer,closed"</formula1>
@@ -4388,6 +4776,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4399,7 +4795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F242"/>
+  <dimension ref="A1:F256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4465,12 +4861,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Manual check required: robots policy unavailable or disallows automated fetch.</t>
+          <t>Robots policy unavailable or disallows automated fetch; not proof the role closed.</t>
         </is>
       </c>
     </row>
@@ -4497,12 +4893,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4529,12 +4925,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Manual check required: robots policy unavailable or disallows automated fetch.</t>
+          <t>Robots policy unavailable or disallows automated fetch; not proof the role closed.</t>
         </is>
       </c>
     </row>
@@ -4561,12 +4957,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Manual check required: robots policy unavailable or disallows automated fetch.</t>
+          <t>Robots policy unavailable or disallows automated fetch; not proof the role closed.</t>
         </is>
       </c>
     </row>
@@ -4593,12 +4989,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Manual check required: robots policy unavailable or disallows automated fetch.</t>
+          <t>Robots policy unavailable or disallows automated fetch; not proof the role closed.</t>
         </is>
       </c>
     </row>
@@ -4625,12 +5021,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4657,12 +5053,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4689,12 +5085,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4721,12 +5117,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4753,12 +5149,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4785,12 +5181,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4817,12 +5213,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Public page fetched; hiring availability still needs employer confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4844,17 +5240,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T15:37:35+00:00</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Manual check required: robots policy unavailable or disallows automated fetch.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -4940,11 +5336,19 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -4964,11 +5368,19 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -4988,11 +5400,19 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -5012,11 +5432,19 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -5036,11 +5464,19 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>blocked</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Exact prior title not found; manual review required, not proof of closure.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -5060,11 +5496,19 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -5084,11 +5528,19 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -7305,12 +7757,12 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Official role detail accessible. Employer listing checked directly and corroborated on company product-team page. Pay undisclosed; hold until stipend confirmed.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -7369,12 +7821,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Official role detail accessible. Full-time early-career role, not an internship. Employer JD and remote-policy careers page were directly read; pay undisclosed.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -7465,12 +7917,12 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Official role detail accessible. Current official board and JD both read. Internship title still asks for shipping experience; do not assume a first-time applicant qualifies. Pay not disclosed.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -7529,12 +7981,12 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Official role detail accessible. Official JD and application form accessible. Remote-first company. Application requires resume, portfolio, start availability, expected monthly stipend and an everyday-app improvement answer. Current stipend not disclosed.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -8324,17 +8776,17 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Search-indexed official page; not directly opened. </t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -8489,12 +8941,12 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Official page opened. </t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9252,17 +9704,17 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>Employer homepage links its YC careers board. Original metadata is from 2024; current intake is unconfirmed. Visible pay says INR 25–40K without a period, while JSON-LD says USD/year; no monthly stipend is confirmed.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9284,17 +9736,17 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>YC board retains this role, originally posted in 2024. Header asks 1+ years, while the body permits current/recent design students and class projects. Employer Join Us currently shows engineering roles. Salary is USD 8–12K/year in structured data, not a monthly INR stipend.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9316,17 +9768,17 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>Indeed detail publicly opened. Three-month UI/UX and web/landing-page internship, in person in Mumbai. Employer careers page confirms company and publishes general HR contact, but this internship was not visible in extracted official openings. Pay/current intake unconfirmed.</t>
+          <t>Public page fetched. Exact prior title not found; manual review required, not proof of closure.</t>
         </is>
       </c>
     </row>
@@ -9348,17 +9800,17 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>Indeed and official careers/role page opened. Explicit Pollachi onsite; remote not assumed. Full-time internship; stipend and posting/closing dates undisclosed.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9380,17 +9832,17 @@
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>Indeed detail publicly opened: Remote India, internship 0–1y. Body dated21 May 2026. CareerScan date3 Oct 2026 repeats the May body; not evidence of a new original posting. Official careers route opened without extractable roles. Verify intake, pay and start window.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9412,17 +9864,17 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>Indeed detail and employer career page opened, both list matching UI/UX Intern0–1. Company Pune-based; specific remote arrangements not confirmed. Stipend/date unknown. Ignore expiry assigned by unrelated mirrors.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9444,17 +9896,17 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>Employer/recruiter-posted Cutshort detail opened. Junior full-time alternative, not internship, asking1–3 years. Listing quotes INR4–6lakh per YEAR; monthly stipend fields must remain null. Work arrangement/current intake require confirmation.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -9476,17 +9928,17 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>Himalayas detail and documented public API both accessible; API per-job check returned200. Detail explicitly permits all countries and API has no country restrictions plus UTC+05:30. Original company site was opened but only ASO/User Acquisition roles were visible, so the UX vacancy is not corroborated on its site. Pay undisclosed. Board labels entry-level while body requires1–2 commercial years.</t>
+          <t>Detail remains available with a 5 November board deadline. The Job expired? control is a report button, not a closure statement.</t>
         </is>
       </c>
     </row>
@@ -11465,12 +11917,12 @@
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>Official detail accessible. Stipend is negotiable with no amount. Careers index advertises immediate joining; later intake is unconfirmed. No remote option. Other company internships have unpaid options, so confirm the design-role policy separately.</t>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
         </is>
       </c>
     </row>
@@ -11492,17 +11944,17 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation.</t>
+          <t>Tracked in295 original removed404/410; archived stable record, application history retained.</t>
         </is>
       </c>
     </row>
@@ -11524,17 +11976,17 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>Employer Dover ATS search index contains role and application fields; direct opening returned a JavaScript shell. Indexed employer copy was crawled about five months before review, not a posting date. Remotive mirror returned403; its relative age does not prove freshness. Pay and duration undisclosed.</t>
+          <t>Public page fetched. Exact prior title not found; manual review required, not proof of closure.</t>
         </is>
       </c>
     </row>
@@ -11940,17 +12392,17 @@
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25T07:18:54+00:00</t>
         </is>
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>Indexed up-to-INR30k listing is expired; upper limit is not a guaranteed minimum.</t>
+          <t>Indeed explicitly expired; up to30k is not a guaranteed minimum.</t>
         </is>
       </c>
     </row>
@@ -11986,8 +12438,456 @@
         </is>
       </c>
     </row>
+    <row r="243" ht="42" customHeight="1">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>Ungrammary</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>https://club.ungrammary.com/jobs/ux%2Fui-trainee-designer</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Public page fetched. Role title found; a fetch alone does not reconfirm intake or compensation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="42" customHeight="1">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Employer detail and application page are available; the form explicitly permits work from home within India. Duration, stipend amount and cohort/start dates are unstated. General employee perks are not confirmed intern benefits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="42" customHeight="1">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>Official careers detail lists JR-045767 and links the Workday application plus a mandatory Microsoft questionnaire. Both steps are required. Workday was not accessible through the research tool; no submission flow tested. Unstop lists 5 November while another mirror gives 7 December; neither is an employer-confirmed deadline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="42" customHeight="1">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS and corporate careers page corroborate this paid job. Unpaid training programs are separate and excluded. Apply through ATS only; the support address is technical support, not a recruitment inbox. Start timing and employment terms need confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="42" customHeight="1">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="42" customHeight="1">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Original Glance Greenhouse role and application are available. Stipend is not stated; the prior StudentSmart INR30–40k/month claim remains unverified. Confirm work arrangement and start date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="42" customHeight="1">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>https://salesforce.wd12.myworkdayjobs.com/en-US/External_Career_Site/job/Summer-2027-Intern---UI-UX-Designer_JR363342</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>Original indexed deadline17 October2026 has passed; fresher mirror dates do not prove renewed intake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="42" customHeight="1">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>Ecolibrium</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ecolibrium.io/careers/</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>Climate/building analytics software. Static careers names UI/UX Intern, but the linked live ATS shows a visual-marketing intern and a product designer requiring3–5 years. No verified current qualifying UX internship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="42" customHeight="1">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>Construe Labs</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>https://construelabs.freshteam.com/jobs/iaTEUebfJP5j/ui-ux-design-intern-remote</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS exposes a three-month UI/UX internship,4–6 hours/day, five days/week. Pay, current intake and India eligibility are not stated. Historical India company evidence does not confirm this intake; watchlist pending clarification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="42" customHeight="1">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>AVYAM LABS</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4829685-ui-ux-designer-intern</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>Original advert explicitly unpaid; excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="42" customHeight="1">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>Entrupy</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4147591-design-intern</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>Indexed internship original now410 Gone; not an active lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="42" customHeight="1">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>MediNex Workforce</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>https://thejobcompany.co.in/frontend/job_details?job_id=6490</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Mirror reports17.5k/month, below remote target; no qualifying card added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="42" customHeight="1">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>CoreByte Studio</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>https://corebytestudio.com/careers/ui-ux-design-intern</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>Remote role explicitly hires within Pakistan, not India.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="42" customHeight="1">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Ecolibrium</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>https://employmenthero.com/jobs/position/ecolibrium-product-designer-72w0q/</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T07:18:54+00:00</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Current product role requires3–5 years; not a junior/internship match.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F242"/>
+  <autoFilter ref="A1:F256"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12060,22 +12960,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>searched</t>
+          <t>Targeted public design search</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Reviewed public design search and selected company job details. Two eligible-region conditional leads retained with older dates and pay caveats. No newly confirmed qualifying monthly stipend. Additional pass: Additional targeted public design/intern search produced no new verified eligible role. Older SuperKalam/Coulomb records remain older listings, not new postings.</t>
+          <t>Public design board and selected details checked. Existing older SuperKalam/Coulomb leads retained with date/pay caveats. No additional newly verified qualifying role.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Public details accessible; applying through YC may require a profile. Company directory is a discovery source, not a vacancy guarantee.</t>
+          <t>Senior and US-only listings excluded; a landing-page listing is not proof of a renewed cohort.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -12093,22 +12993,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>limited</t>
+          <t>Targeted indexed search</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Direct filtered route was not accessible in the research tool; public YC employer pages provide overlapping job content. Additional pass: Additional targeted public design/intern search produced no new verified eligible role. Older SuperKalam/Coulomb records remain older listings, not new postings.</t>
+          <t>India design-intern search performed alongside YC board review; no additional eligible detail verified.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Do not double-count YC and Work at a Startup mirrors as different openings.</t>
+          <t>Public targeted sample, not an exhaustive database crawl.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -12126,22 +13026,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>searched</t>
+          <t>API scan and targeted review</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Fetched the actual October2026 thread via Algolia API:266 top-level posts,25 mentioning designer/UX/design-engineer terms. No verified India-eligible UX/product internship or junior role from this pass. Cardog and Sundream retained as conditional company targets. Additional pass: Additional Algolia API scan of266 top-level comments: strict designer/UX/UI/product-design terms matched20 (different methodology from prior25-term count). No additional paid India-eligible junior design internship verified.</t>
+          <t>October thread Algolia API again returned266 top-level comments;20 strict design/UX/UI term matches. Sampled matching posts did not yield another verified India-eligible paid UX/product internship or junior vacancy.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Engineering, senior, North-America/Europe-only and volunteer posts were not promoted as qualifying design internships.</t>
+          <t>Strict term matching differs from the older25-term count; engineering, senior, volunteer and restricted-geography posts are not recommendations.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -12192,22 +13092,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Public details and search results accessible</t>
+          <t>Public details and targeted search</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Expanded targeted searches beyond four earlier listings. Four new relevant details retained with undisclosed stipend (Icogz, VictorFlow, Balusen, Gunadhya), plus genuine cross-post enrichments. Numerous other interns are below pay floor, unpaid, wrong discipline or expired; no inference that search counts equal relevant vacancies. Additional pass: Additional targeted check: BiCSoM fresher detail opened, but old original/closed LinkedIn makes it watchlist-only; Melento minimum INR11k is below target; Kixar and Redliner copies expired. No new qualifying Indeed vacancy added.</t>
+          <t>Existing Indeed detail pages rechecked. Icogz title corrected to original Intern-UI/UX without changing ID. Redliner explicitly expired; low pay and misleading maximum-only claims excluded. No additional qualifying Indeed-primary role added.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Search sample, not the entire inventory; current pay remains unstated unless original advert says otherwise.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -12229,7 +13129,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -12239,12 +13139,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Direct/domain public queries again reported robots restrictions. No newly verified original Naukri role; existing employer-linked route retained. Account connection was not tested or required for these public-source checks; do not imply signed-in access. Additional pass: Targeted public queries again blocked by robots; no original or signed-in access verified and no new role invented.</t>
+          <t>Targeted original/domain search again blocked or inaccessible; no new original vacancy verified. Existing employer-linked route retained.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>No signed-in account access or bypass used.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -12262,22 +13162,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Public role details accessible; apply uses candidate login</t>
+          <t>Targeted public search</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Qoruz junior product UX alternative found with annual pay preserved; Ungrammary matching internship adds below-target advertised pay context. Monsoonfish/Integra/AMPM below target and unrelated Product Management roles excluded. Current public examples were mostly below target: Integra Magna INR 3–5k/month, AMPM INR 10–15k/month, SDS INR 7–15k/month. BigThinkCode has an annual INR 1–3 lakh header and restrictive cohort/certification requirements, retained as company research. Ungrammary cross-post adds an annual range and inactive-recruiter caveat to an existing role. Additional pass: Additional targeted public search/category sample yielded no new independently verified qualifying UX/product internship or fresher detail. Coverage is sampled; no claim that all listings were searched.</t>
+          <t>Current-looking results included Integra Magna3–5k/month and Monsoonfish5–10k/month, below target. No source quota filled with unsuitable cards.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Original monthly ranges kept distinct from annual salary and aggregator maxima.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -12336,22 +13236,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Blocked by robots.txt</t>
+          <t>Restricted public access</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Public domain search reported robots restriction. No new original role verified; no CAPTCHA bypass or signed-in session attempted. Additional pass: Additional public domain queries again robots-blocked; no original session or access-control bypass attempted.</t>
+          <t>Direct public UI/UX route unavailable through research tool. No original details verified in this pass.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>No authenticated access or blanket freshness claim.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -12369,22 +13269,22 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Targeted public search only</t>
+          <t>Targeted indexed search</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Targeted indexed design-intern/0–1 year queries produced no independently verified eligible detail in this pass. This is a coverage limitation, not proof of no jobs; authenticated matching workflow not inspected. Additional pass: Additional targeted public search/category sample yielded no new independently verified qualifying UX/product internship or fresher detail. Coverage is sampled; no claim that all listings were searched.</t>
+          <t>Design-intern site query did not produce a newly verified eligible detail in this pass.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>No original/authenticated inventory inspection established.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -12402,22 +13302,22 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Partial public coverage; originals individually checked</t>
+          <t>Original details checked; stale indexes flagged</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Several indexed internships were expired on direct check; accessible ads often unpaid or below target. Attira preserved as company/conditional research, no proven qualifying stipend. Accounts may be needed to apply/save, not to research these public detail pages. Additional pass: BetterStory remote INR25k visual internship detail opened; employer explicitly excludes product/UX scope, so not shortlisted.</t>
+          <t>Entrupy and Chiblu4209561 originals now410. Chiblu employer page remains separate evidence and record stays on hold. AVYAM and Ourora unpaid; BetterStory outside UX/product scope. No suitable new verified vacancy added.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Indexed cards may survive removed originals. Header compensation periods must not be guessed.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -12439,22 +13339,22 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Public API and individual details checked</t>
+          <t>Existing detail rechecked and targeted search</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Documented public API checks: India product-designer internships returned 0; UX internships returned 6, including five developer/graphic roles and GWEN fee-based training. Entry-level UI/UX search returned 6 records: one plausible junior opening at Energise.pro, an experienced Cloud Counselage role, a GitLab talent pool, adjacent QA and graphic roles. Category counts alone do not establish suitable vacancies. Additional pass: Additional targeted public search/category sample yielded no new independently verified qualifying UX/product internship or fresher detail. Coverage is sampled; no claim that all listings were searched.</t>
+          <t>Energise.pro listing still states worldwide, one-year minimum and5 November board deadline. Job expired? is a report button. No new suitable internship verified.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Full-time junior alternative remains on hold for commercial experience/pay/employer intake; no automatic closure from report controls.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -12476,22 +13376,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Public category opened; sample checked</t>
+          <t>Targeted public search</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>No suitable India-eligible UX/product internship or fresher role verified in the examined public sample. Visible roles were predominantly senior/principal/manager or geographically restricted. Category-level Anywhere in the World labels are insufficient evidence of country eligibility. Additional pass: Additional targeted public search/category sample yielded no new independently verified qualifying UX/product internship or fresher detail. Coverage is sampled; no claim that all listings were searched.</t>
+          <t>Reviewed indexed design/contract results and Construelabs company page. No new verified full-time India-eligible junior/intern product role. LooseGrip part-time contract not established as an eligible internship.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>General worldwide labels can conflict with title/office geography; individual detail verification required.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -12513,22 +13413,22 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Public listing/category checked; limited role detail</t>
+          <t>Targeted indexed search</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>No suitable India-eligible UX/product internship or junior role verified from examined categories and junior filters. A junior brand-design example was Canada-only; a worldwide junior graphic role was outside the requested discipline. Additional pass: Additional targeted public search/category sample yielded no new independently verified qualifying UX/product internship or fresher detail. Coverage is sampled; no claim that all listings were searched.</t>
+          <t>Search surfaced worker profiles rather than suitable employer details; no new role accepted.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Worker profiles are people seeking work, not vacancies.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -12550,22 +13450,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Indexed leads with employer corroboration; mirror details403/404</t>
+          <t>Targeted public search</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Opened design, India andinternpublicpages. No suitable UX/product internship or junior role verified; visible examples were geographic restrictions, senior, graphic/video or other disciplines. Did not bypass paid access or promise comprehensive coverage. Additional pass: Unitedover mirror403 and Innovexis mirror404. Innovexis employer-hosted in295 detail accessible with undisclosed amount; Unitedover employer Dover index only, direct JS shell. Both kept on hold with separate verification limits; mirror relative dates are not original posting dates.</t>
+          <t>Trackier graphic-design intern surfaced; broad marketing/video scope not promoted as a focused UX/product role. Unitedover prior lead retained with original intake limits.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>No new confirmed stipend or fresh-original assertion.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -12587,22 +13487,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Public category opened; sample checked</t>
+          <t>Targeted public search</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Examined public designcategory. Product/visual roles predominantly US-national orUSlocal/hybrid; no suitable Indiaeligibleintern/junior verified. Additional pass: Additional targeted public search/category sample yielded no new independently verified qualifying UX/product internship or fresher detail. Coverage is sampled; no claim that all listings were searched.</t>
+          <t>India design search surfaced experienced sound-design work outside requested discipline; no qualifying new role verified.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Targeted indexed sample only.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -12624,22 +13524,22 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Alternate public category opened; no eligible detail verified</t>
+          <t>Direct route inaccessible; targeted search limited</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Design URL could not be accessed and targetedpublicsearch yielded no independently verifiable matching detail. This is an access/coverage gap, not evidence of no jobs. Additional pass: Alternate /remote-entry-level-product-design-jobs page opened. No new India-eligible internship/junior employer detail verified; index/category labels alone do not establish experience or geography.</t>
+          <t>Design route could not be opened through research tool; cross-board indexed search yielded no verified new matching detail.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Do not claim full board inspection.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
@@ -12690,22 +13590,22 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Public employer directory inspected</t>
+          <t>Attempted directory route; unavailable</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Accessible India startup directory includes existing targets such as Swiggy, Meesho, Groww and Juspay. Rankings/funding do not establish an active business, stipend or design vacancy; verify official careers. Additional pass: Public discovery page reopened; no vacancy inferred from map membership or funding/rank. Role acceptance still requires employer/job-detail evidence.</t>
+          <t>The /startups/india route returned404. No vacancy inferred from directory membership.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Best-effort public targeted sample; original dates, intake and eligibility are verified only where explicitly documented.</t>
+          <t>Employer discovery only; do not claim an entire map was inspected.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
@@ -12789,22 +13689,22 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Targeted public checks</t>
+          <t>Employer/ATS research and existing-lead recheck</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>New Arihant AI and Innovexis employer-hosted internships have undisclosed pay; Unitedover indexed employer ATS remains current-intake unverified. Parallel internship archived; BiCSoM historical fresher page is watchlist-only.</t>
+          <t>Rechecked all39 existing primary URLs subject to robots/access limits:34 pages fetched,4 blocked and1 original removed. New Atlabs/Revvity internships and Moonfire/Enterprise Bot fresher jobs; Glance upgraded to original Greenhouse. Innovexis in295 archived. Ecolibrium stale-careers discrepancy recorded.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Public sample only; no exhaustive or authenticated access claim.</t>
+          <t>A fetched page alone is not proof of active intake. Stipend, cohort dates and office terms remain held where unstated.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -12822,22 +13722,22 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Targeted public checks</t>
+          <t>Public indexed search; no new verified original</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Targeted indexed UX/product/interaction internship searches produced no newly independently verified original X hiring post. Existing Wint/BThree crossposts retained; no claim of original authenticated access.</t>
+          <t>Targeted India UX/product internship searches produced no newly independently verified original post. Earlier Wint/BThree crossposts retained.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Public sample only; no exhaustive or authenticated access claim.</t>
+          <t>No signed-in X session; zero new verified results does not imply no vacancies exist.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -12855,22 +13755,22 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Targeted public checks</t>
+          <t>Targeted public search and corroboration</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Targeted early-career searches used as corroboration. BiCSoM crosspost explicitly closed; no new LinkedIn-primary role added. Relative ages are not verified original posting dates.</t>
+          <t>Revvity employer crosspost enriches the same new official role, not a duplicate. BNP remote advert is four months old with amount/current intake unverified; not promoted as newly active. Generic/low-pay listings not added for source quotas.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Public sample only; no exhaustive or authenticated access claim.</t>
+          <t>Relative ages and discovery dates are distinct from original publication dates.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
@@ -12887,7 +13787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M116"/>
+  <dimension ref="A1:M124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -18363,7 +19263,7 @@
       </c>
       <c r="M114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -18461,8 +19361,384 @@
         </is>
       </c>
     </row>
+    <row r="117" ht="42" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Suggested employer target based on a published early-career role; no hiring probability implied.</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="n"/>
+      <c r="G117" s="2" t="n"/>
+      <c r="H117" s="2" t="inlineStr"/>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Remote-India product-design internship on AI video workflows. Employer offers a competitive stipend without an amount.</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr"/>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="42" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Suggested employer target based on a published early-career role; no hiring probability implied.</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="n"/>
+      <c r="G118" s="2" t="n"/>
+      <c r="H118" s="2" t="inlineStr"/>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>Life-sciences software UX internship spanning research and design. Stipend, duration and intake timing require confirmation.</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="42" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Suggested employer target based on a published early-career role; no hiring probability implied.</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="n"/>
+      <c r="G119" s="2" t="n"/>
+      <c r="H119" s="2" t="inlineStr"/>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>Paid permanent fresher alternative, not an internship. Original salary is INR 2.5–4 lakh per year.</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="42" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Suggested employer target based on a published early-career role; no hiring probability implied.</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="n"/>
+      <c r="G120" s="2" t="n"/>
+      <c r="H120" s="2" t="inlineStr"/>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>Permanent early-career UI/product-interface role, not an internship. Pay is absent from the original employer ATS.</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="42" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Published UX internship; pay and intake still need confirmation.</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr"/>
+      <c r="F121" s="2" t="n"/>
+      <c r="G121" s="2" t="n"/>
+      <c r="H121" s="2" t="inlineStr"/>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>No employer-stated amount; aggregator INR30–40k/month is unverified.</t>
+        </is>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t>https://glance.com/careers/latest</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr"/>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="42" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Summer2027 M.Des class-of2027 role. Original indexed deadline17 October has passed despite later mirror dates; no current card added. Check for reopened cohorts.</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="n"/>
+      <c r="G122" s="2" t="n"/>
+      <c r="H122" s="2" t="inlineStr"/>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>No current qualifying stipend established</t>
+        </is>
+      </c>
+      <c r="K122" s="3" t="inlineStr">
+        <is>
+          <t>https://salesforce.wd12.myworkdayjobs.com/en-US/External_Career_Site/job/Summer-2027-Intern---UI-UX-Designer_JR363342</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="42" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Ecolibrium</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Climate/building analytics software. Static careers names UI/UX Intern, but the linked live ATS shows a visual-marketing intern and a product designer requiring3–5 years. No verified current qualifying UX internship.</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr"/>
+      <c r="F123" s="2" t="n"/>
+      <c r="G123" s="2" t="n"/>
+      <c r="H123" s="2" t="inlineStr"/>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>No current qualifying stipend established</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ecolibrium.io/careers/</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="42" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Construe Labs</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS exposes a three-month UI/UX internship,4–6 hours/day, five days/week. Pay, current intake and India eligibility are not stated. Historical India company evidence does not confirm this intake; watchlist pending clarification.</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="n"/>
+      <c r="G124" s="2" t="n"/>
+      <c r="H124" s="2" t="inlineStr"/>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>No current qualifying stipend established</t>
+        </is>
+      </c>
+      <c r="K124" s="3" t="inlineStr">
+        <is>
+          <t>https://construelabs.freshteam.com/jobs/iaTEUebfJP5j/ui-ux-design-intern-remote</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M116"/>
+  <autoFilter ref="A1:M124"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Dream,Workable,Possible"</formula1>
@@ -18602,6 +19878,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L114" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K123" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId141"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18613,7 +19897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M116"/>
+  <dimension ref="A1:M124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -25686,7 +26970,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Advertised internship; pay and intake require confirmation</t>
+          <t>Tracked in295 role removed; company target retained without an active-vacancy claim</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -25717,7 +27001,7 @@
       </c>
       <c r="M114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -25847,8 +27131,456 @@
         </is>
       </c>
     </row>
+    <row r="117" ht="42" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>AI video creation software</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>Remote within India; Gurugram office optional/preferred</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Advertised role; eligibility, pay and intake need review</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr"/>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern/apply</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>Published application route</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr"/>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="42" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>Life-sciences technology and software</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>Thane / Mumbai, Maharashtra; employer pages use both locations</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Advertised role; eligibility, pay and intake need review</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>https://revvity.wd103.myworkdayjobs.com/External/job/Mumbai/UX-Intern_JR-045767/apply</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>Published application route</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="42" customHeight="1">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Services / technology group</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>Business software and technology services</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>Advertised role; eligibility, pay and intake need review</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr"/>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/apply.php?job_id=50</t>
+        </is>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>Published application route</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="42" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>Conversational AI and enterprise automation</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Advertised role; eligibility, pay and intake need review</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>Published application route</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="42" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>AI shopping and television experiences</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; remote eligibility not stated</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>Official UX internship detail and application available</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>https://glance.com/careers/latest</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
+        </is>
+      </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>Official application</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr"/>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="42" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Summer2027 M</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Watchlist only; no qualifying current vacancy confirmed</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>https://salesforce.wd12.myworkdayjobs.com/en-US/External_Career_Site/job/Summer-2027-Intern---UI-UX-Designer_JR363342</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr"/>
+      <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="42" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Ecolibrium</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>Climate/building analytics software</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>Watchlist only; no qualifying current vacancy confirmed</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ecolibrium.io/careers/</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr"/>
+      <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="42" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Construe Labs</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Services company</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS exposes a three-month UI/UX internship,4–6 hours/day, five days/week</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Remote; current country eligibility unstated</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Watchlist only; no qualifying current vacancy confirmed</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>https://construelabs.freshteam.com/jobs/iaTEUebfJP5j/ui-ux-design-intern-remote</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M116"/>
+  <autoFilter ref="A1:M124"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
@@ -26065,6 +27797,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J115" r:id="rId213"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J116" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J117" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H118" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J118" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H119" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J119" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J120" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J121" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId228"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26076,7 +27821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I179"/>
+  <dimension ref="A1:I203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -33389,7 +35134,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation.</t>
+          <t>Original in295 role removed (404/410) on25 October2026; retained for history.</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -33432,7 +35177,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation.</t>
+          <t>Original in295 role removed (404/410) on25 October2026; retained for history.</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -33475,7 +35220,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation.</t>
+          <t>Original in295 role removed (404/410) on25 October2026; retained for history.</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -33518,7 +35263,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>Employer-hosted ATS detail accessible. Mentions annual compensation without a figure; no monthly stipend established. Relative publication ages vary across indexed copies and are not reliable original dates. A different older same-company ATS listing advertises INR20–25k/month, below the remote target; it does not set this listing’s pay. Employer also sells training; employment terms and absence of fees need confirmation.</t>
+          <t>Original in295 role removed (404/410) on25 October2026; retained for history.</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -33791,8 +35536,1040 @@
       </c>
       <c r="I179" s="2" t="inlineStr"/>
     </row>
+    <row r="180" ht="42" customHeight="1">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>Remote within India; Gurugram office optional/preferred</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Employer detail and application page are available; the form explicitly permits work from home within India. Duration, stipend amount and cohort/start dates are unstated. General employee perks are not confirmed intern benefits.</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>Figma proficiency and a portfolio showing design reasoning</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr"/>
+    </row>
+    <row r="181" ht="42" customHeight="1">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Remote within India; Gurugram office optional/preferred</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Employer detail and application page are available; the form explicitly permits work from home within India. Duration, stipend amount and cohort/start dates are unstated. General employee perks are not confirmed intern benefits.</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>Interface fundamentals, interaction flows and usability</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr"/>
+    </row>
+    <row r="182" ht="42" customHeight="1">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Remote within India; Gurugram office optional/preferred</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Employer detail and application page are available; the form explicitly permits work from home within India. Duration, stipend amount and cohort/start dates are unstated. General employee perks are not confirmed intern benefits.</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>Independent ownership and collaboration with engineering</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr"/>
+    </row>
+    <row r="183" ht="42" customHeight="1">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>Atlabs</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Remote within India; Gurugram office optional/preferred</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>https://join.atlabs.ai/roles/product-design-intern</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>Employer detail and application page are available; the form explicitly permits work from home within India. Duration, stipend amount and cohort/start dates are unstated. General employee perks are not confirmed intern benefits.</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>Interest in AI creative tools; prior product work is optional</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr"/>
+    </row>
+    <row r="184" ht="42" customHeight="1">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Thane / Mumbai, Maharashtra; employer pages use both locations</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>Official careers detail lists JR-045767 and links the Workday application plus a mandatory Microsoft questionnaire. Both steps are required. Workday was not accessible through the research tool; no submission flow tested. Unstop lists 5 November while another mirror gives 7 December; neither is an employer-confirmed deadline.</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>Awareness of UX design and research methods</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr"/>
+    </row>
+    <row r="185" ht="42" customHeight="1">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>Thane / Mumbai, Maharashtra; employer pages use both locations</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>Official careers detail lists JR-045767 and links the Workday application plus a mandatory Microsoft questionnaire. Both steps are required. Workday was not accessible through the research tool; no submission flow tested. Unstop lists 5 November while another mirror gives 7 December; neither is an employer-confirmed deadline.</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>Clear English communication and presenting design decisions</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr"/>
+    </row>
+    <row r="186" ht="42" customHeight="1">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Thane / Mumbai, Maharashtra; employer pages use both locations</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>Official careers detail lists JR-045767 and links the Workday application plus a mandatory Microsoft questionnaire. Both steps are required. Workday was not accessible through the research tool; no submission flow tested. Unstop lists 5 November while another mirror gives 7 December; neither is an employer-confirmed deadline.</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>Curiosity, feedback and collaboration</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr"/>
+    </row>
+    <row r="187" ht="42" customHeight="1">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>Revvity</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>UX Intern</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Thane / Mumbai, Maharashtra; employer pages use both locations</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.revvity.com/job/thane/ux-intern/20539/102245859808</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>Official careers detail lists JR-045767 and links the Workday application plus a mandatory Microsoft questionnaire. Both steps are required. Workday was not accessible through the research tool; no submission flow tested. Unstop lists 5 November while another mirror gives 7 December; neither is an employer-confirmed deadline.</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>Work includes prototyping and research sessions</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr"/>
+    </row>
+    <row r="188" ht="42" customHeight="1">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>UI / UX Design Trainee (Fresher)</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS and corporate careers page corroborate this paid job. Unpaid training programs are separate and excluded. Apply through ATS only; the support address is technical support, not a recruitment inbox. Start timing and employment terms need confirmation.</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>Design, HCI, fine-arts or related qualification</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr"/>
+    </row>
+    <row r="189" ht="42" customHeight="1">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>UI / UX Design Trainee (Fresher)</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS and corporate careers page corroborate this paid job. Unpaid training programs are separate and excluded. Apply through ATS only; the support address is technical support, not a recruitment inbox. Start timing and employment terms need confirmation.</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>Working Figma knowledge and a portfolio; coursework is accepted</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr"/>
+    </row>
+    <row r="190" ht="42" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>UI / UX Design Trainee (Fresher)</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS and corporate careers page corroborate this paid job. Unpaid training programs are separate and excluded. Apply through ATS only; the support address is technical support, not a recruitment inbox. Start timing and employment terms need confirmation.</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>Wireframes, design-system components and research support</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr"/>
+    </row>
+    <row r="191" ht="42" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Moonfire</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>UI / UX Design Trainee (Fresher)</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>https://ats.moonfiregroup.com/jobs/ui-ux-design-trainee-fresher</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS and corporate careers page corroborate this paid job. Unpaid training programs are separate and excluded. Apply through ATS only; the support address is technical support, not a recruitment inbox. Start timing and employment terms need confirmation.</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>Openness to critique</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr"/>
+    </row>
+    <row r="192" ht="42" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>UI Designer – 0–1 Years Experience</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>0–1 years; graduates with a portfolio are welcome</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr"/>
+    </row>
+    <row r="193" ht="42" customHeight="1">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>UI Designer – 0–1 Years Experience</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>Figma and strong typography, spacing, grids and interface hierarchy</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr"/>
+    </row>
+    <row r="194" ht="42" customHeight="1">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>UI Designer – 0–1 Years Experience</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>Basic UX knowledge and responsive SaaS interfaces</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr"/>
+    </row>
+    <row r="195" ht="42" customHeight="1">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>UI Designer – 0–1 Years Experience</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>Collaboration, iteration and curiosity about AI tools</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr"/>
+    </row>
+    <row r="196" ht="42" customHeight="1">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise Bot</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>UI Designer – 0–1 Years Experience</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>Junior / fresher</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru; ATS says hybrid but also five days/week on-site</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/enterprisebot/16830986-ui-designer-0-1-years-experience</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>JOIN employer detail advertises 45 hours/week, six-month probation and ASAP start. Hybrid header conflicts with five on-site days. A mirror advertises INR30–50k/month, which the original does not confirm; no verified stipend is inferred.</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>Bonus: design systems, HTML/CSS and prior design internship</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr"/>
+    </row>
+    <row r="197" ht="42" customHeight="1">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>Official role accessible; pay/intake unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>Design student or recent graduate with a portfolio showing reasoning and craft</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr"/>
+    </row>
+    <row r="198" ht="42" customHeight="1">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Official role accessible; pay/intake unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>Interaction and system thinking for TV shopping experiences</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr"/>
+    </row>
+    <row r="199" ht="42" customHeight="1">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>Official role accessible; pay/intake unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>Design-system patterns, iteration and engineering handoff</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr"/>
+    </row>
+    <row r="200" ht="42" customHeight="1">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7916115</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Official role accessible; pay/intake unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Interest in AI or large-screen products is optional</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr"/>
+    </row>
+    <row r="201" ht="42" customHeight="1">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Summer2027 Intern - UI/UX Designer</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Expired cohort evidence</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hyderabad</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>https://salesforce.wd12.myworkdayjobs.com/en-US/External_Career_Site/job/Summer-2027-Intern---UI-UX-Designer_JR363342</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Summer2027 M.Des class-of2027 role. Original indexed deadline17 October has passed despite later mirror dates; no current card added. Check for reopened cohorts.</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr"/>
+    </row>
+    <row r="202" ht="42" customHeight="1">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Ecolibrium</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Intern</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Unverified current intake</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ecolibrium.io/careers/</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>Climate/building analytics software. Static careers names UI/UX Intern, but the linked live ATS shows a visual-marketing intern and a product designer requiring3–5 years. No verified current qualifying UX internship.</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr"/>
+    </row>
+    <row r="203" ht="42" customHeight="1">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Construe Labs</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern (Remote)</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>Part-time internship; intake/geography unconfirmed</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>Remote; current country eligibility unstated</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>https://construelabs.freshteam.com/jobs/iaTEUebfJP5j/ui-ux-design-intern-remote</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>Employer ATS exposes a three-month UI/UX internship,4–6 hours/day, five days/week. Pay, current intake and India eligibility are not stated. Historical India company evidence does not confirm this intake; watchlist pending clarification.</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I179"/>
+  <autoFilter ref="A1:I203"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Unassessed,Met,Partly met,Gap"</formula1>
@@ -33977,6 +36754,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E203" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33988,7 +36789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -34003,7 +36804,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Research snapshot: 2026-10-24</t>
+          <t>Research snapshot: 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -34784,6 +37585,90 @@
       <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Historical2022 role with a still-accessible form, but LinkedIn crosspost closed; watchlist only pending a new intake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="42" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>AVYAM LABS</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Original advert explicitly unpaid; excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="42" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Entrupy</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Indexed internship original now410 Gone; not an active lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="42" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Original indexed deadline17 October2026 has passed; fresher mirror dates do not prove renewed intake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="42" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>MediNex Workforce</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Mirror reports17.5k/month, below remote target; no qualifying card added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="42" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>CoreByte Studio</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Remote role explicitly hires within Pakistan, not India.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="42" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Ecolibrium</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Current product role requires3–5 years; not a junior/internship match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="42" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Innovexis</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Tracked in295 original removed404/410; archived stable record, application history retained.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add verified startup design internship research and source caveats
</commit_message>
<xml_diff>
--- a/topics/job-search-agent/app/public/data/internships.xlsx
+++ b/topics/job-search-agent/app/public/data/internships.xlsx
@@ -16,12 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$Z$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$F$256</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source coverage'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Company watchlist'!$A$1:$M$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Company directory'!$A$1:$M$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Role requirements'!$A$1:$I$203</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internships'!$A$1:$Z$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$F$273</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source coverage'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Company watchlist'!$A$1:$M$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Company directory'!$A$1:$M$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Role requirements'!$A$1:$I$226</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z44"/>
+  <dimension ref="A1:Z48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4690,8 +4690,400 @@
       </c>
       <c r="Z44" s="2" t="inlineStr"/>
     </row>
+    <row r="45" ht="95" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Design Intern</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Remote or Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Confirm paid status, monthly stipend, duration and joining window; review AI/mobile-design expectations.</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern?apply=1</t>
+        </is>
+      </c>
+      <c r="R45" s="2" t="inlineStr"/>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>Published employer form/contact; manual review</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio; student or personal projects accepted; Figma components, responsive layouts and design systems; Practical AI-assisted design and an interest in funnel analysis; Android/Material conventions and ability to iterate quickly</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="inlineStr"/>
+      <c r="W45" s="2" t="inlineStr">
+        <is>
+          <t>Employer posting date not stated; newly researched, not newly posted</t>
+        </is>
+      </c>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="95" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Remote; Ahmedabad-based product team, India</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Confirm stipend, hours, India work arrangement and a suitable 3–4 month duration; use the employer internship form.</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="R46" s="2" t="inlineStr"/>
+      <c r="S46" s="2" t="inlineStr">
+        <is>
+          <t>Published employer form/contact; manual review</t>
+        </is>
+      </c>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>Figma, prototyping, user research and design-system skills named; Interest in student-editor and faculty-dashboard usability; Clarify hours and duration before proceeding</t>
+        </is>
+      </c>
+      <c r="V46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="inlineStr">
+        <is>
+          <t>Employer posting date not stated; newly researched, not newly posted</t>
+        </is>
+      </c>
+      <c r="X46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="95" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Remote Global / Singapore; confirm India contracting and hours</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Confirm paid status, monthly amount, duration, India engagement and time-zone overlap before applying.</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="Q47" s="3" t="inlineStr">
+        <is>
+          <t>mailto:careers@formas.ai</t>
+        </is>
+      </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>careers@formas.ai</t>
+        </is>
+      </c>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>Published employer form/contact; manual review</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>Design/HCI/interaction-design student or recent graduate; Figma familiarity and interface-design fundamentals; Prototyping, component-library work and usability-test support</t>
+        </is>
+      </c>
+      <c r="V47" s="2" t="inlineStr">
+        <is>
+          <t>Employer requests portfolio, resume and a short note about design technology and AI.</t>
+        </is>
+      </c>
+      <c r="W47" s="2" t="inlineStr">
+        <is>
+          <t>Employer posting date not stated; newly researched, not newly posted</t>
+        </is>
+      </c>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="95" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; UI/UX Intern</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>On-site</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>on_hold</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Confirm compensation, eligibility and start window through the published careers contact before proceeding.</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>Company careers</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>mailto:daankart.com@gmail.com</t>
+        </is>
+      </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>daankart.com@gmail.com</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="inlineStr">
+        <is>
+          <t>Published employer form/contact; manual review</t>
+        </is>
+      </c>
+      <c r="T48" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>Figma comfort and user-journey thinking; Explain design decisions and work with engineering; Research, prototyping and usability testing; Design for trust and conversion; six-month office commitment</t>
+        </is>
+      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>Published careers contact for the Hyderabad product/UI internship; confirm paid terms before sending an application.</t>
+        </is>
+      </c>
+      <c r="W48" s="2" t="inlineStr">
+        <is>
+          <t>Employer posting date not stated; newly researched, not newly posted</t>
+        </is>
+      </c>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Y48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="Z48" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z44"/>
+  <autoFilter ref="A1:Z48"/>
   <dataValidations count="1">
     <dataValidation sqref="J2:J10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"discovered,shortlisted,on_hold,applied,assessment,interview,offer,closed"</formula1>
@@ -4784,6 +5176,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4795,7 +5195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F256"/>
+  <dimension ref="A1:F273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -12886,8 +13286,552 @@
         </is>
       </c>
     </row>
+    <row r="257" ht="42" customHeight="1">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="42" customHeight="1">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="42" customHeight="1">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="42" customHeight="1">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="42" customHeight="1">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>Coachingle</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>https://www.coachingle.com/careers</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Official product role requires3+ years, confirmed in the public role-description bundle. Company target only, not an intern/junior recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="42" customHeight="1">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Cravv</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4716470-product-design-intern</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Employer Wellfound detail lists20k/month and digital/device work. Below the non-Gujarat target; retain as a watchlist-only company, not a qualifying new job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="42" customHeight="1">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>Figr</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>https://careers.antler.co/companies/figr/jobs/48650001-product-design-intern</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Antler original detail explicitly says no longer accepting. Current opening not inferred from a stale search snippet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="42" customHeight="1">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>Grexa AI</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>https://peerlist.io/company/grexa_ai/careers/product-design-intern/jobhlknq7lkradbbdc7dbmeg9ne98p</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Original Peerlist employer post is archived; watch for a renewed role rather than treating it as current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="42" customHeight="1">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>Globalli</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>https://globalli.io/company/careers</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>Current official linked Greenhouse API exposes13 jobs and no designer role. Mirrored junior descriptions remain unverified; no active card added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="42" customHeight="1">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>Superteams.ai</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>https://www.superteams.ai/career/figma-design-intern/</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Original role explicitly closed despite its listing on the general careers index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" ht="42" customHeight="1">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>Leap</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>https://leapfinance.freshteam.com/jobs/sTgwRD31WhNQ/product-design-intern</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>Original ATS host/detail returns a site-not-found page; indexed internship not confirmed current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="42" customHeight="1">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>LeelaRam Technologies</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>https://www.leelaramtechnologies.com/careers/ui-ux-design-intern</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>Original stipend10–15k/month in Mumbai, below target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="42" customHeight="1">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>GoPratle</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4555222-ui-ux-intern-remote-clone</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>Original header2–5k and final-year/fresher restriction; not a qualifying stipend match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="42" customHeight="1">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4029436-product-design-intern</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>Original410 Gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="42" customHeight="1">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>frover</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/3307361-product-designer-intern-ui-ux</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>Original410 Gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="42" customHeight="1">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Mowka</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4503290-product-designer-intern</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>Original410 Gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="42" customHeight="1">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>eLeoRex Technologies</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>https://eleorex.com/about-us/career/ui-ux-design-intern/</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T16:54:39+00:00</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>Original1October2026 deadline passed; not a current internship recommendation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F256"/>
+  <autoFilter ref="A1:F273"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12898,7 +13842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -13775,8 +14719,45 @@
       </c>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Startup design hiring</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Targeted original-role and startup-board checks</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Four new on-hold startup internships:Propel, Kodin/Autometa Labs, FORMAS.AI and Daankart. Six existing startup leads tagged for search, without duplicate job cards. Added missing employer-directory records and five caveated company targets. Figr/Grexa/Superteams closed, Leap original unavailable, Coachingle experienced-only, Globalli no current ATS designer role; low-pay roles excluded. No new qualifying monthly stipend confirmed.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Best-effort employer, Wellfound, Peerlist, Antler and public search sample. Newly discovered does not mean newly posted. Remote Global still requires India contracting/time-zone confirmation. Startup stage/funding is not independently audited.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Superteams.ai: Original role explicitly closed despite its listing on the general careers index.; Leap: Original ATS host/detail returns a site-not-found page; indexed internship not confirmed current.; LeelaRam Technologies: Original stipend10–15k/month in Mumbai, below target.; GoPratle: Original header2–5k and final-year/fresher restriction; not a qualifying stipend match.; FLIP: Original410 Gone.; frover: Original410 Gone.; Mowka: Original410 Gone.; eLeoRex Technologies: Original1October2026 deadline passed; not a current internship recommendation.; Figr: Antler original detail explicitly says no longer accepting. Current opening not inferred from a stale search snippet.; Grexa AI: Original Peerlist employer post is archived; watch for a renewed role rather than treating it as current.; Cravv: Employer Wellfound detail lists20k/month and digital/device work. Below the non-Gujarat target; retain as a watchlist-only company, not a qualifying new job.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13787,7 +14768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M124"/>
+  <dimension ref="A1:M137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -19737,8 +20718,619 @@
         </is>
       </c>
     </row>
+    <row r="125" ht="42" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="n"/>
+      <c r="G125" s="2" t="n"/>
+      <c r="H125" s="2" t="inlineStr"/>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>Design app interfaces, systems and growth assets at an AI-focused consumer-app team. Full-time internship. Amount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="K125" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="42" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr"/>
+      <c r="F126" s="2" t="n"/>
+      <c r="G126" s="2" t="n"/>
+      <c r="H126" s="2" t="inlineStr"/>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>Design student-editor and faculty-dashboard experiences. Employer lists a 2–4 month internship with flexible start. Amount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="K126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="42" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr"/>
+      <c r="F127" s="2" t="n"/>
+      <c r="G127" s="2" t="n"/>
+      <c r="H127" s="2" t="inlineStr"/>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>Prototype and improve a spatial-design product, including interface components and usability testing. Amount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="42" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="n"/>
+      <c r="G128" s="2" t="n"/>
+      <c r="H128" s="2" t="inlineStr"/>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>Research and improve donor journeys, interface consistency and a component library. Six-month, full-time office internship. Amount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="K128" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="42" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>RevRag AI</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Original employer advert already researched today; stipend and intake terms remain unconfirmed.</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr"/>
+      <c r="F129" s="2" t="n"/>
+      <c r="G129" s="2" t="n"/>
+      <c r="H129" s="2" t="inlineStr"/>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.revrag.ai/careers/product-design-intern</t>
+        </is>
+      </c>
+      <c r="L129" s="2" t="inlineStr"/>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="42" customHeight="1">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>NeuralPath Technologies</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Original employer advert already researched today; stipend and intake terms remain unconfirmed.</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr"/>
+      <c r="F130" s="2" t="n"/>
+      <c r="G130" s="2" t="n"/>
+      <c r="H130" s="2" t="inlineStr"/>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.neuralpath.app/careers/</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr"/>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="42" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Zavio</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Original employer advert already researched today; stipend and intake terms remain unconfirmed.</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr"/>
+      <c r="F131" s="2" t="n"/>
+      <c r="G131" s="2" t="n"/>
+      <c r="H131" s="2" t="inlineStr"/>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gozavio.com/careers</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr"/>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="42" customHeight="1">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Chiblu</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Existing researched role; stipend and renewed intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="n"/>
+      <c r="G132" s="2" t="n"/>
+      <c r="H132" s="2" t="inlineStr"/>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K132" s="3" t="inlineStr">
+        <is>
+          <t>https://chiblu.com/careers/product-design-intern-ux-ui</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr"/>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="42" customHeight="1">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Coachingle</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>Official product role requires3+ years, confirmed in the public role-description bundle. Company target only, not an intern/junior recommendation.</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr"/>
+      <c r="F133" s="2" t="n"/>
+      <c r="G133" s="2" t="n"/>
+      <c r="H133" s="2" t="inlineStr"/>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.coachingle.com/careers</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr"/>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="42" customHeight="1">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Cravv</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Employer Wellfound detail lists20k/month and digital/device work. Below the non-Gujarat target; retain as a watchlist-only company, not a qualifying new job.</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="n"/>
+      <c r="G134" s="2" t="n"/>
+      <c r="H134" s="2" t="inlineStr"/>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>Employer advert:INR20,000/month, below the non-Gujarat target; not a current offer to the applicant.</t>
+        </is>
+      </c>
+      <c r="K134" s="3" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4716470-product-design-intern</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr"/>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="42" customHeight="1">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Figr</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Antler original detail explicitly says no longer accepting. Current opening not inferred from a stale search snippet.</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr"/>
+      <c r="F135" s="2" t="n"/>
+      <c r="G135" s="2" t="n"/>
+      <c r="H135" s="2" t="inlineStr"/>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K135" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.antler.co/companies/figr/jobs/48650001-product-design-intern</t>
+        </is>
+      </c>
+      <c r="L135" s="2" t="inlineStr"/>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="42" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Grexa AI</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Original Peerlist employer post is archived; watch for a renewed role rather than treating it as current.</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="n"/>
+      <c r="G136" s="2" t="n"/>
+      <c r="H136" s="2" t="inlineStr"/>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K136" s="3" t="inlineStr">
+        <is>
+          <t>https://peerlist.io/company/grexa_ai/careers/product-design-intern/jobhlknq7lkradbbdc7dbmeg9ne98p</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="42" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Globalli</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Current official linked Greenhouse API exposes13 jobs and no designer role. Mirrored junior descriptions remain unverified; no active card added.</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Not established</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr"/>
+      <c r="F137" s="2" t="n"/>
+      <c r="G137" s="2" t="n"/>
+      <c r="H137" s="2" t="inlineStr"/>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying current stipend established unless explicitly stated in role evidence.</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr">
+        <is>
+          <t>https://globalli.io/company/careers</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M124"/>
+  <autoFilter ref="A1:M137"/>
   <dataValidations count="1">
     <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Dream,Workable,Possible"</formula1>
@@ -19886,6 +21478,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K123" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K125" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K126" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId154"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19897,7 +21502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M124"/>
+  <dimension ref="A1:M137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -27579,8 +29184,775 @@
         </is>
       </c>
     </row>
+    <row r="125" ht="42" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>Consumer-app publishing and product growth</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>Remote or Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="42" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Education software and coding-lab interfaces</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>Remote; Ahmedabad-based product team, India</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr"/>
+      <c r="J126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="42" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>AI design software for architecture and interiors</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>Remote Global / Singapore; confirm India contracting and hours</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="42" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Donation and crowdfunding product software</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="42" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>RevRag AI</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>AI agents for financial workflows</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Original employer advert already researched today; stipend and intake terms remain unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.revrag.ai/careers/product-design-intern</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.revrag.ai/careers/product-design-intern</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L129" s="2" t="inlineStr"/>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="42" customHeight="1">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>NeuralPath Technologies</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Privacy-first consumer applications</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Remote, India</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Original employer advert already researched today; stipend and intake terms remain unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.neuralpath.app/careers/</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.neuralpath.app/careers/</t>
+        </is>
+      </c>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr"/>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="42" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Zavio</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Workable</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Financial education software</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>Remote, India</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Original employer advert already researched today; stipend and intake terms remain unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gozavio.com/careers</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gozavio.com/careers</t>
+        </is>
+      </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr"/>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="42" customHeight="1">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Chiblu</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Marketplace software for independent makers</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>Remote, India; Bengaluru preferred</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Existing researched role; stipend and renewed intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="inlineStr">
+        <is>
+          <t>https://chiblu.com/careers/product-design-intern-ux-ui</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr">
+        <is>
+          <t>https://chiblu.com/careers/product-design-intern-ux-ui</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr"/>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="42" customHeight="1">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Coachingle</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>AI learning software</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>Remote India</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Official product role requires3+ years, confirmed in the public role-description bundle. Company target only, not an intern/junior recommendation.</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.coachingle.com/careers</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.coachingle.com/careers</t>
+        </is>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr"/>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="42" customHeight="1">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Cravv</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>AI cooking device and companion app</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, office; six months</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Employer Wellfound detail lists20k/month and digital/device work. Below the non-Gujarat target; retain as a watchlist-only company, not a qualifying new job.</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H134" s="3" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4716470-product-design-intern</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4716470-product-design-intern</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr"/>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="42" customHeight="1">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Figr</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>AI product-design tools</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru / remote historical description</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Antler original detail explicitly says no longer accepting. Current opening not inferred from a stale search snippet.</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H135" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.antler.co/companies/figr/jobs/48650001-product-design-intern</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.antler.co/companies/figr/jobs/48650001-product-design-intern</t>
+        </is>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L135" s="2" t="inlineStr"/>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="42" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Grexa AI</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>AI marketing software</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>Navi Mumbai, office</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Original Peerlist employer post is archived; watch for a renewed role rather than treating it as current.</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H136" s="3" t="inlineStr">
+        <is>
+          <t>https://peerlist.io/company/grexa_ai/careers/product-design-intern/jobhlknq7lkradbbdc7dbmeg9ne98p</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr">
+        <is>
+          <t>https://peerlist.io/company/grexa_ai/careers/product-design-intern/jobhlknq7lkradbbdc7dbmeg9ne98p</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="42" customHeight="1">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Globalli</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Product company</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Workforce-management software</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>Indexed remote India/Pakistan; current intake unconfirmed</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Current official linked Greenhouse API exposes13 jobs and no designer role. Mirrored junior descriptions remain unverified; no active card added.</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>UX Designer; Product Designer; Interaction Designer</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="inlineStr">
+        <is>
+          <t>https://globalli.io/company/careers</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr">
+        <is>
+          <t>https://globalli.io/company/careers</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Published careers/application route</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M124"/>
+  <autoFilter ref="A1:M137"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
@@ -27810,6 +30182,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H122" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H123" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J125" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J126" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J127" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J130" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J131" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J132" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J133" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J134" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J135" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J136" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J137" r:id="rId254"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27821,7 +30219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I203"/>
+  <dimension ref="A1:I226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -36568,8 +38966,997 @@
       </c>
       <c r="I203" s="2" t="inlineStr"/>
     </row>
+    <row r="204" ht="42" customHeight="1">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>Design Intern</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Remote or Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>Portfolio; student or personal projects accepted</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr"/>
+    </row>
+    <row r="205" ht="42" customHeight="1">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>Design Intern</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>Remote or Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>Figma components, responsive layouts and design systems</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr"/>
+    </row>
+    <row r="206" ht="42" customHeight="1">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>Design Intern</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>Remote or Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>Practical AI-assisted design and an interest in funnel analysis</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr"/>
+    </row>
+    <row r="207" ht="42" customHeight="1">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Propel</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Design Intern</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>Remote or Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>https://gopropel.in/careers/design-intern/</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>Rendered official detail verified, including interface work and AI-assisted iteration. Stipend, duration and start dates are unstated. This is not a confirmed paid-stipend match.</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>Android/Material conventions and ability to iterate quickly</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr"/>
+    </row>
+    <row r="208" ht="42" customHeight="1">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>Remote; Ahmedabad-based product team, India</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Figma, prototyping, user research and design-system skills named</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr"/>
+    </row>
+    <row r="209" ht="42" customHeight="1">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>Remote; Ahmedabad-based product team, India</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>Interest in student-editor and faculty-dashboard usability</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr"/>
+    </row>
+    <row r="210" ht="42" customHeight="1">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>Kodin / Autometa Labs</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>Remote; Ahmedabad-based product team, India</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>https://www.getkodin.com/#careers</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Official careers section advertises a stipend without an amount. It names Figma, prototypes, research and design systems; no formal degree or experience requirement is stated. Hours and intake need confirmation.</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>Clarify hours and duration before proceeding</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr"/>
+    </row>
+    <row r="211" ht="42" customHeight="1">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>Remote Global / Singapore; confirm India contracting and hours</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>Design/HCI/interaction-design student or recent graduate</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr"/>
+    </row>
+    <row r="212" ht="42" customHeight="1">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Remote Global / Singapore; confirm India contracting and hours</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>Figma familiarity and interface-design fundamentals</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr"/>
+    </row>
+    <row r="213" ht="42" customHeight="1">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>FORMAS.AI</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>UI/UX Design Intern</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Remote Global / Singapore; confirm India contracting and hours</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>https://www.formas.ai/careers</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>Specific internship detail says Remote Global / Singapore and allows full-time or part-time work. Current design/HCI students or recent graduates are eligible in the advert. Pay, duration and local engagement terms are unstated.</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>Prototyping, component-library work and usability-test support</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr"/>
+    </row>
+    <row r="214" ht="42" customHeight="1">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; UI/UX Intern</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>Figma comfort and user-journey thinking</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr"/>
+    </row>
+    <row r="215" ht="42" customHeight="1">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; UI/UX Intern</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>Explain design decisions and work with engineering</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr"/>
+    </row>
+    <row r="216" ht="42" customHeight="1">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; UI/UX Intern</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>Research, prototyping and usability testing</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr"/>
+    </row>
+    <row r="217" ht="42" customHeight="1">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Daankart</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; UI/UX Intern</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>https://daankart.com/about/careers#open-roles</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>Official careers page names the role, location, duration and HR contact. Stipend and exact start window are not stated; do not infer a paid offer from internship benefits.</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>Design for trust and conversion; six-month office commitment</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr"/>
+    </row>
+    <row r="218" ht="42" customHeight="1">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>RevRag AI</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>https://www.revrag.ai/careers/product-design-intern</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>Original company role is accessible and lists Bengaluru on-site. Third-party ₹40k claims are not confirmed by this page.</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr"/>
+    </row>
+    <row r="219" ht="42" customHeight="1">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>NeuralPath Technologies</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>Remote, India</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>https://www.neuralpath.app/careers/</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>Company careers page explicitly lists a remote Product Design Intern opportunity and year-round applications. Duration and stipend are discussed individually.</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr"/>
+    </row>
+    <row r="220" ht="42" customHeight="1">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>Zavio</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Remote, India</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gozavio.com/careers</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>Company careers page lists this as an open internship, remote anywhere in India. Stipend and posting date are not stated.</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr"/>
+    </row>
+    <row r="221" ht="42" customHeight="1">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>Chiblu</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern (UX &amp; UI)</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>Remote, India; Bengaluru preferred</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>https://chiblu.com/careers/product-design-intern-ux-ui</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>Company still exposes the role page and links it from careers. It is an older May posting; current hiring and stipend require confirmation. Recheck25 October: employer page remains accessible; linked Wellfound4209561 now returns410 Gone. The employer page alone does not establish a renewed intake.</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr"/>
+    </row>
+    <row r="222" ht="42" customHeight="1">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>Coachingle</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Product Designer</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>Experienced; 3+ years</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Remote India</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>https://www.coachingle.com/careers</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>Official product role requires3+ years, confirmed in the public role-description bundle. Company target only, not an intern/junior recommendation.</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr"/>
+    </row>
+    <row r="223" ht="42" customHeight="1">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>Cravv</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>Internship; below pay target</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, office; six months</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>https://wellfound.com/jobs/4716470-product-design-intern</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>Employer Wellfound detail lists20k/month and digital/device work. Below the non-Gujarat target; retain as a watchlist-only company, not a qualifying new job.</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr"/>
+    </row>
+    <row r="224" ht="42" customHeight="1">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>Figr</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>Closed internship evidence</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru / remote historical description</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.antler.co/companies/figr/jobs/48650001-product-design-intern</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>Antler original detail explicitly says no longer accepting. Current opening not inferred from a stale search snippet.</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr"/>
+    </row>
+    <row r="225" ht="42" customHeight="1">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>Grexa AI</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>Product Design Intern</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>Archived internship evidence</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>Navi Mumbai, office</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>https://peerlist.io/company/grexa_ai/careers/product-design-intern/jobhlknq7lkradbbdc7dbmeg9ne98p</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Original Peerlist employer post is archived; watch for a renewed role rather than treating it as current.</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr"/>
+    </row>
+    <row r="226" ht="42" customHeight="1">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Globalli</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Junior Product Designer</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>Indexed historical lead</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>Indexed remote India/Pakistan; current intake unconfirmed</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>https://globalli.io/company/careers</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Current official linked Greenhouse API exposes13 jobs and no designer role. Mirrored junior descriptions remain unverified; no active card added.</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>No detailed requirements captured; open source</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>Unassessed</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I203"/>
+  <autoFilter ref="A1:I226"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Unassessed,Met,Partly met,Gap"</formula1>
@@ -36778,6 +40165,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E201" r:id="rId200"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E202" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E226" r:id="rId225"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -36789,7 +40199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -37672,6 +41082,138 @@
         </is>
       </c>
     </row>
+    <row r="74" ht="42" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Superteams.ai</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Original role explicitly closed despite its listing on the general careers index.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="42" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Leap</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Original ATS host/detail returns a site-not-found page; indexed internship not confirmed current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="42" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>LeelaRam Technologies</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Original stipend10–15k/month in Mumbai, below target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="42" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>GoPratle</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Original header2–5k and final-year/fresher restriction; not a qualifying stipend match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="42" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>FLIP</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Original410 Gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="42" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>frover</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Original410 Gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="42" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Mowka</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Original410 Gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="42" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>eLeoRex Technologies</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Original1October2026 deadline passed; not a current internship recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="42" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Figr</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Antler original detail explicitly says no longer accepting. Current opening not inferred from a stale search snippet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="42" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Grexa AI</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Original Peerlist employer post is archived; watch for a renewed role rather than treating it as current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="42" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Cravv</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Employer Wellfound detail lists20k/month and digital/device work. Below the non-Gujarat target; retain as a watchlist-only company, not a qualifying new job.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>